<commit_message>
DataBases: added diagram for idef1x
</commit_message>
<xml_diff>
--- a/Data Analysis/LW4/betterLife.xlsx
+++ b/Data Analysis/LW4/betterLife.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\archive\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\studies\Data Analysis\LW4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1132EF07-AC11-4572-865E-8E6A522D78E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6BCE432-5C83-4AAF-A49A-E22A7C09A489}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="611" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="622" uniqueCount="262">
   <si>
     <t>Country</t>
   </si>
@@ -832,6 +832,9 @@
   </si>
   <si>
     <t>Xср</t>
+  </si>
+  <si>
+    <t>Исходная матрица</t>
   </si>
 </sst>
 </file>
@@ -1162,13 +1165,6 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <bottom style="thin">
-          <color theme="9" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
         <left style="thin">
           <color theme="9" tint="0.39997558519241921"/>
         </left>
@@ -1184,10 +1180,75 @@
       </border>
     </dxf>
     <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="9" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="9" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="9" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="9" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="9" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -1345,78 +1406,10 @@
       </border>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="9" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="9" tint="0.39997558519241921"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="9" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="9" tint="0.39997558519241921"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
       <border outline="0">
         <top style="thin">
           <color theme="9" tint="0.39997558519241921"/>
         </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="9" tint="0.39997558519241921"/>
-        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -1434,6 +1427,16 @@
           <color theme="9" tint="0.39997558519241921"/>
         </bottom>
       </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="9" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1558,23 +1561,23 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{97CED990-E0AD-4049-9D5C-9EDAE3A0398E}" name="Таблица2" displayName="Таблица2" ref="A1:G39" totalsRowShown="0" headerRowDxfId="11" headerRowBorderDxfId="20" tableBorderDxfId="21" totalsRowBorderDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{97CED990-E0AD-4049-9D5C-9EDAE3A0398E}" name="Таблица2" displayName="Таблица2" ref="A1:G39" totalsRowShown="0" headerRowDxfId="21" headerRowBorderDxfId="20" tableBorderDxfId="19" totalsRowBorderDxfId="18">
   <autoFilter ref="A1:G39" xr:uid="{97CED990-E0AD-4049-9D5C-9EDAE3A0398E}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{804D964C-0E40-443F-8354-7E3A6A793E82}" name="Country" dataDxfId="18"/>
+    <tableColumn id="1" xr3:uid="{804D964C-0E40-443F-8354-7E3A6A793E82}" name="Country" dataDxfId="17"/>
     <tableColumn id="4" xr3:uid="{9D470B8E-97B5-4D07-A7CD-6F42A4DAC2B3}" name="GDP per capita (USD)" dataDxfId="16"/>
     <tableColumn id="7" xr3:uid="{5CD4D351-DDBF-41AD-9297-7129B9BA1A82}" name="  Life expectancy" dataDxfId="15"/>
     <tableColumn id="5" xr3:uid="{FF20AAFF-E8B0-4F26-84F8-B4D77D4CCDC0}" name="  Employment rate" dataDxfId="14"/>
     <tableColumn id="6" xr3:uid="{38326172-D301-4B95-B35D-E9E32D23F670}" name="  Quality of support network" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{76A806F8-1375-4D41-B135-FF8715BCA6CE}" name="  Feeling safe walking alone at night" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{B8AE9B68-9413-4263-A7EF-480763C86177}" name="  Life satisfaction" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{76A806F8-1375-4D41-B135-FF8715BCA6CE}" name="  Feeling safe walking alone at night" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{B8AE9B68-9413-4263-A7EF-480763C86177}" name="  Life satisfaction" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A73368B3-40A2-41F3-AD78-5390C5A50577}" name="Таблица24" displayName="Таблица24" ref="I1:O39" totalsRowShown="0" headerRowDxfId="10" headerRowBorderDxfId="8" tableBorderDxfId="9" totalsRowBorderDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A73368B3-40A2-41F3-AD78-5390C5A50577}" name="Таблица24" displayName="Таблица24" ref="I1:O39" totalsRowShown="0" headerRowDxfId="10" headerRowBorderDxfId="9" tableBorderDxfId="8" totalsRowBorderDxfId="7">
   <autoFilter ref="I1:O39" xr:uid="{A73368B3-40A2-41F3-AD78-5390C5A50577}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{F84D075D-1627-48E2-B085-6D6223B23906}" name="Country" dataDxfId="6"/>
@@ -4965,10 +4968,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O41"/>
+  <dimension ref="A1:O53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="18.140625" customWidth="1"/>
     <col min="2" max="2" width="16.7109375" customWidth="1"/>
     <col min="3" max="3" width="14.7109375" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
@@ -6955,6 +6958,149 @@
       <c r="G41">
         <f>AVERAGE(Таблица2[[  Life satisfaction]])</f>
         <v>6.6868421052631595</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>261</v>
+      </c>
+      <c r="B44" t="s">
+        <v>26</v>
+      </c>
+      <c r="C44">
+        <v>2.0157894736841939</v>
+      </c>
+      <c r="D44">
+        <v>4.3421052631578902</v>
+      </c>
+      <c r="E44">
+        <v>1.9210526315789451</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B45" t="s">
+        <v>38</v>
+      </c>
+      <c r="C45">
+        <v>1.0157894736841939</v>
+      </c>
+      <c r="D45">
+        <v>3.3421052631578902</v>
+      </c>
+      <c r="E45">
+        <v>0.92105263157894512</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B46" t="s">
+        <v>62</v>
+      </c>
+      <c r="C46">
+        <v>1.1157894736841882</v>
+      </c>
+      <c r="D46">
+        <v>1.3421052631578902</v>
+      </c>
+      <c r="E46">
+        <v>1.9210526315789451</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B47" t="s">
+        <v>102</v>
+      </c>
+      <c r="C47">
+        <v>0.51578947368419392</v>
+      </c>
+      <c r="D47">
+        <v>5.3421052631578902</v>
+      </c>
+      <c r="E47">
+        <v>3.9210526315789451</v>
+      </c>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B48" t="s">
+        <v>120</v>
+      </c>
+      <c r="C48">
+        <v>1.9157894736841996</v>
+      </c>
+      <c r="D48">
+        <v>-3.6578947368421098</v>
+      </c>
+      <c r="E48">
+        <v>2.9210526315789451</v>
+      </c>
+    </row>
+    <row r="49" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B49" t="s">
+        <v>125</v>
+      </c>
+      <c r="C49">
+        <v>0.41578947368419961</v>
+      </c>
+      <c r="D49">
+        <v>8.3421052631578902</v>
+      </c>
+      <c r="E49">
+        <v>-1.0789473684210549</v>
+      </c>
+    </row>
+    <row r="50" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B50" t="s">
+        <v>210</v>
+      </c>
+      <c r="C50">
+        <v>2.0157894736841939</v>
+      </c>
+      <c r="D50">
+        <v>6.3421052631578902</v>
+      </c>
+      <c r="E50">
+        <v>4.9210526315789451</v>
+      </c>
+    </row>
+    <row r="51" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B51" t="s">
+        <v>241</v>
+      </c>
+      <c r="C51">
+        <v>3.0157894736841939</v>
+      </c>
+      <c r="D51">
+        <v>11.34210526315789</v>
+      </c>
+      <c r="E51">
+        <v>2.9210526315789451</v>
+      </c>
+    </row>
+    <row r="52" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B52" t="s">
+        <v>252</v>
+      </c>
+      <c r="C52">
+        <v>0.31578947368419108</v>
+      </c>
+      <c r="D52">
+        <v>6.3421052631578902</v>
+      </c>
+      <c r="E52">
+        <v>1.9210526315789451</v>
+      </c>
+    </row>
+    <row r="53" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B53" t="s">
+        <v>256</v>
+      </c>
+      <c r="C53">
+        <v>-2.0842105263158004</v>
+      </c>
+      <c r="D53">
+        <v>-1.6578947368421098</v>
+      </c>
+      <c r="E53">
+        <v>2.9210526315789451</v>
       </c>
     </row>
   </sheetData>

</xml_diff>